<commit_message>
fix(mock-data): add missing Teachers tab to import fixture
The fixture predates the Teachers tab being made required (tab-schema.ts
REQUIRED_TABS), so it fails workbook-parser's tab-presence check. Added
8 rows reusing the same teacher/class pairs already present in the
Classes and Users tabs, each with a subject and class-teacher flag.
</commit_message>
<xml_diff>
--- a/infra/mock-data/school-connect-mock-import.xlsx
+++ b/infra/mock-data/school-connect-mock-import.xlsx
@@ -9,13 +9,14 @@
     <sheet sheetId="3" name="Users" state="visible" r:id="rId6"/>
     <sheet sheetId="4" name="Students" state="visible" r:id="rId7"/>
     <sheet sheetId="5" name="Fee Structures" state="visible" r:id="rId8"/>
+    <sheet sheetId="6" name="Teachers" state="visible" r:id="rId9"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1245" uniqueCount="737">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1308" uniqueCount="747">
   <si>
     <t>School Connect — Bulk Onboarding Template</t>
   </si>
@@ -2226,6 +2227,36 @@
   </si>
   <si>
     <t>2025-12-15</t>
+  </si>
+  <si>
+    <t>Teacher Name*</t>
+  </si>
+  <si>
+    <t>Phone Number*</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>Subject Name*</t>
+  </si>
+  <si>
+    <t>Is Class Teacher</t>
+  </si>
+  <si>
+    <t>Mathematics</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Science</t>
+  </si>
+  <si>
+    <t>English</t>
+  </si>
+  <si>
+    <t>Social Studies</t>
   </si>
 </sst>
 </file>
@@ -7124,4 +7155,230 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G9"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="20" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="3" width="28" customWidth="1"/>
+    <col min="4" max="4" width="14" customWidth="1"/>
+    <col min="5" max="5" width="10" customWidth="1"/>
+    <col min="6" max="7" width="16" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>737</v>
+      </c>
+      <c r="B1" t="s">
+        <v>738</v>
+      </c>
+      <c r="C1" t="s">
+        <v>739</v>
+      </c>
+      <c r="D1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E1" t="s">
+        <v>724</v>
+      </c>
+      <c r="F1" t="s">
+        <v>740</v>
+      </c>
+      <c r="G1" t="s">
+        <v>741</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F2" t="s">
+        <v>742</v>
+      </c>
+      <c r="G2" t="s">
+        <v>743</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F3" t="s">
+        <v>744</v>
+      </c>
+      <c r="G3" t="s">
+        <v>743</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>46</v>
+      </c>
+      <c r="B4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F4" t="s">
+        <v>745</v>
+      </c>
+      <c r="G4" t="s">
+        <v>743</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>48</v>
+      </c>
+      <c r="B5" t="s">
+        <v>49</v>
+      </c>
+      <c r="C5" t="s">
+        <v>27</v>
+      </c>
+      <c r="D5" t="s">
+        <v>26</v>
+      </c>
+      <c r="E5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F5" t="s">
+        <v>746</v>
+      </c>
+      <c r="G5" t="s">
+        <v>743</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B6" t="s">
+        <v>51</v>
+      </c>
+      <c r="C6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D6" t="s">
+        <v>28</v>
+      </c>
+      <c r="E6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F6" t="s">
+        <v>742</v>
+      </c>
+      <c r="G6" t="s">
+        <v>743</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>52</v>
+      </c>
+      <c r="B7" t="s">
+        <v>53</v>
+      </c>
+      <c r="C7" t="s">
+        <v>31</v>
+      </c>
+      <c r="D7" t="s">
+        <v>30</v>
+      </c>
+      <c r="E7" t="s">
+        <v>19</v>
+      </c>
+      <c r="F7" t="s">
+        <v>744</v>
+      </c>
+      <c r="G7" t="s">
+        <v>743</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>54</v>
+      </c>
+      <c r="B8" t="s">
+        <v>55</v>
+      </c>
+      <c r="C8" t="s">
+        <v>33</v>
+      </c>
+      <c r="D8" t="s">
+        <v>32</v>
+      </c>
+      <c r="E8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F8" t="s">
+        <v>745</v>
+      </c>
+      <c r="G8" t="s">
+        <v>743</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>56</v>
+      </c>
+      <c r="B9" t="s">
+        <v>57</v>
+      </c>
+      <c r="C9" t="s">
+        <v>35</v>
+      </c>
+      <c r="D9" t="s">
+        <v>34</v>
+      </c>
+      <c r="E9" t="s">
+        <v>19</v>
+      </c>
+      <c r="F9" t="s">
+        <v>746</v>
+      </c>
+      <c r="G9" t="s">
+        <v>743</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
 </file>
</xml_diff>